<commit_message>
feat: attach master raw and clean excel data workbook and add 5-year revenue trajectory
</commit_message>
<xml_diff>
--- a/documentation/kpi_reconciliation.xlsx
+++ b/documentation/kpi_reconciliation.xlsx
@@ -473,14 +473,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
-    <col width="43" customWidth="1" min="2" max="2"/>
-    <col width="43" customWidth="1" min="3" max="3"/>
-    <col width="43" customWidth="1" min="4" max="4"/>
-    <col width="43" customWidth="1" min="5" max="5"/>
+    <col width="47" customWidth="1" min="2" max="2"/>
+    <col width="47" customWidth="1" min="3" max="3"/>
+    <col width="47" customWidth="1" min="4" max="4"/>
+    <col width="47" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -533,22 +533,22 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>61,926</t>
+          <t>66,019</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>61,926</t>
+          <t>66,019</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>61,926</t>
+          <t>66,019</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>61,926</t>
+          <t>66,019</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -565,22 +565,22 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>19,021</t>
+          <t>20,056</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>19,021</t>
+          <t>20,056</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>19,021</t>
+          <t>20,056</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>19,021</t>
+          <t>20,056</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -597,22 +597,22 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>11,500</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>11,500</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>11,500</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>11,500</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -725,22 +725,22 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>₹45,828,146.55</t>
+          <t>₹48,818,717.05</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>₹45,828,146.55</t>
+          <t>₹48,818,717.05</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>₹45,828,146.55</t>
+          <t>₹48,818,717.05</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>₹45,828,146.55</t>
+          <t>₹48,818,717.05</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -757,22 +757,22 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>77,567</t>
+          <t>82,873</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>77,567</t>
+          <t>82,873</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>77,567</t>
+          <t>82,873</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>77,567</t>
+          <t>82,873</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -789,22 +789,22 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>₹2,409.34</t>
+          <t>₹2,434.12</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>₹2,409.34</t>
+          <t>₹2,434.12</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>₹2,409.34</t>
+          <t>₹2,434.12</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>₹2,409.34</t>
+          <t>₹2,434.12</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -821,22 +821,22 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>4,047</t>
+          <t>4,248</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>4,047</t>
+          <t>4,248</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>4,047</t>
+          <t>4,248</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>4,047</t>
+          <t>4,248</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -853,22 +853,22 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>35.19%</t>
+          <t>35.40%</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>35.19%</t>
+          <t>35.40%</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>35.19%</t>
+          <t>35.40%</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>35.19%</t>
+          <t>35.40%</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -885,22 +885,22 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>₹17,316,104.20</t>
+          <t>₹18,444,504.79</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>₹17,316,104.20</t>
+          <t>₹18,444,504.79</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>₹17,316,104.20</t>
+          <t>₹18,444,504.79</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>₹17,316,104.20</t>
+          <t>₹18,444,504.79</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -981,22 +981,22 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>₹12,389,744.40</t>
+          <t>₹13,205,918.55</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>₹12,389,744.40</t>
+          <t>₹13,205,918.55</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>₹12,389,744.40</t>
+          <t>₹13,205,918.55</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>₹12,389,744.40</t>
+          <t>₹13,205,918.55</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -1045,22 +1045,22 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>₹11,515,055.25</t>
+          <t>₹12,276,789.35</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>₹11,515,055.25</t>
+          <t>₹12,276,789.35</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>₹11,515,055.25</t>
+          <t>₹12,276,789.35</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>₹11,515,055.25</t>
+          <t>₹12,276,789.35</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1077,22 +1077,22 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>25.13%</t>
+          <t>25.15%</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>25.13%</t>
+          <t>25.15%</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>25.13%</t>
+          <t>25.15%</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>25.13%</t>
+          <t>25.15%</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1109,57 +1109,25 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>JBL Computer Peripheral V84 (PRD-1092)</t>
+          <t>Zebronics Smart Home Device V15 (PRD-1071)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>JBL Computer Peripheral V84 (PRD-1092)</t>
+          <t>Zebronics Smart Home Device V15 (PRD-1071)</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>JBL Computer Peripheral V84 (PRD-1092)</t>
+          <t>Zebronics Smart Home Device V15 (PRD-1071)</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>JBL Computer Peripheral V84 (PRD-1092)</t>
+          <t>Zebronics Smart Home Device V15 (PRD-1071)</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>Revenue Growth (YoY)</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>162.98%</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>162.98%</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>162.98%</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>162.98%</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1221,7 +1189,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>61,926 Transactions</t>
+          <t>66,019 Transactions</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1238,7 +1206,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>11,500 Customers</t>
+          <t>12,000 Customers</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1306,7 +1274,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>₹4.58 Crore (₹45,828,146.55)</t>
+          <t>₹4.88 Crore (₹48,818,717.05)</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1323,7 +1291,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>₹2,409.34</t>
+          <t>₹2,434.12</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1340,7 +1308,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>35.19% (4,047 customers)</t>
+          <t>35.40% (4,248 customers)</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1357,7 +1325,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Electronics (₹12,389,744.40 - 27.04%)</t>
+          <t>Electronics (₹13,205,918.55 - 27.05%)</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1374,7 +1342,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>West (25.13%)</t>
+          <t>West (25.15%)</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1425,7 +1393,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>8 Actionable RFM Segments across 11,500 users</t>
+          <t>8 Actionable RFM Segments across 12,000 users</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">

</xml_diff>